<commit_message>
Cap daily picks to max 2 top stocks and enforce 100% deterministic symbol tie-breaking
</commit_message>
<xml_diff>
--- a/data/trade_ledger.xlsx
+++ b/data/trade_ledger.xlsx
@@ -484,12 +484,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X2"/>
+  <dimension ref="A1:X4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="33" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="R2" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="S2" s="7" t="n">
         <v>-1.28</v>
@@ -715,7 +715,175 @@
       <c r="W2" s="2" t="inlineStr"/>
       <c r="X2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 19:19:09</t>
+          <t>2026-08-16 19:50:48</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>REC-20260816-UBL-4BC2FA</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>UBL</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>United Breweries Limited</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>83.8</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>1376.6</v>
+      </c>
+      <c r="I3" s="3" t="n">
+        <v>1394.51</v>
+      </c>
+      <c r="J3" s="3" t="n">
+        <v>1306.54</v>
+      </c>
+      <c r="K3" s="3" t="n">
+        <v>1552.86</v>
+      </c>
+      <c r="L3" s="3" t="n">
+        <v>1640.83</v>
+      </c>
+      <c r="M3" s="3" t="n">
+        <v>1790.38</v>
+      </c>
+      <c r="N3" s="2" t="n">
+        <v>113</v>
+      </c>
+      <c r="O3" s="3" t="n">
+        <v>157579.63</v>
+      </c>
+      <c r="P3" s="3" t="n">
+        <v>1376.6</v>
+      </c>
+      <c r="Q3" s="6" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="R3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="S3" s="7" t="n">
+        <v>-1.28</v>
+      </c>
+      <c r="T3" s="3" t="n">
+        <v>-2023.83</v>
+      </c>
+      <c r="U3" s="2" t="inlineStr"/>
+      <c r="V3" s="2" t="inlineStr"/>
+      <c r="W3" s="2" t="inlineStr"/>
+      <c r="X3" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-16 19:50:48</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>REC-20260816-ABBOTINDIA-D586CC</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>ABBOTINDIA</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Abbott India Limited</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>83.8</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>27060</v>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>27412.1</v>
+      </c>
+      <c r="J4" s="3" t="n">
+        <v>25546</v>
+      </c>
+      <c r="K4" s="3" t="n">
+        <v>30771.08</v>
+      </c>
+      <c r="L4" s="3" t="n">
+        <v>32637.18</v>
+      </c>
+      <c r="M4" s="3" t="n">
+        <v>35809.55</v>
+      </c>
+      <c r="N4" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="O4" s="3" t="n">
+        <v>137060.5</v>
+      </c>
+      <c r="P4" s="3" t="n">
+        <v>27060</v>
+      </c>
+      <c r="Q4" s="6" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="R4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="S4" s="7" t="n">
+        <v>-1.28</v>
+      </c>
+      <c r="T4" s="3" t="n">
+        <v>-1760.5</v>
+      </c>
+      <c r="U4" s="2" t="inlineStr"/>
+      <c r="V4" s="2" t="inlineStr"/>
+      <c r="W4" s="2" t="inlineStr"/>
+      <c r="X4" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-16 19:50:48</t>
         </is>
       </c>
     </row>

</xml_diff>